<commit_message>
fix(templates): align numeric insets across budget sheets
</commit_message>
<xml_diff>
--- a/public/downloads/plantillas-um-sans/2026.10.09-r3/presupuesto-interno.xlsx
+++ b/public/downloads/plantillas-um-sans/2026.10.09-r3/presupuesto-interno.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultado" sheetId="1" r:id="R8edb85e8ab5d4f55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costeo" sheetId="2" r:id="Rf8356f98c8bf44e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parámetros" sheetId="3" r:id="Recf42a5a56aa4c97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proveedores" sheetId="4" r:id="R70ddaee43c2342fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultado" sheetId="1" r:id="Reb7885532b654d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costeo" sheetId="2" r:id="R3fb5afca74f5464a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parámetros" sheetId="3" r:id="R80b17b0d63424fa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proveedores" sheetId="4" r:id="R016a30933d22414f"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Resultado'!$A$1:$F$28</x:definedName>
@@ -24,13 +24,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="10">
     <x:numFmt numFmtId="200" formatCode="dd/mm/yyyy"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.00;(#,##0.00);0.00"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
     <x:numFmt numFmtId="203" formatCode="@"/>
     <x:numFmt numFmtId="204" formatCode="0.##"/>
     <x:numFmt numFmtId="205" formatCode="General;General;General;@_W"/>
+    <x:numFmt numFmtId="206" formatCode="#,##0.00_W;(#,##0.00)_W;0.00_W;@_W"/>
+    <x:numFmt numFmtId="207" formatCode="0.##_W"/>
+    <x:numFmt numFmtId="208" formatCode="0.0%_W"/>
+    <x:numFmt numFmtId="209" formatCode="General_W"/>
   </x:numFmts>
   <x:fonts count="10">
     <x:font>
@@ -451,8 +455,8 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" horizontal="left" indent="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
+    <x:xf numFmtId="206" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" indent="1"/>
@@ -460,8 +464,8 @@
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" horizontal="left" indent="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
+    <x:xf numFmtId="206" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" indent="1"/>
@@ -469,8 +473,8 @@
     <x:xf numFmtId="201" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" indent="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
+    <x:xf numFmtId="206" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" horizontal="left" indent="1"/>
@@ -478,8 +482,8 @@
     <x:xf numFmtId="201" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" indent="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
+    <x:xf numFmtId="206" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1" indent="0"/>
@@ -493,20 +497,20 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" horizontal="center" indent="0"/>
     </x:xf>
-    <x:xf numFmtId="204" fontId="7" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
+    <x:xf numFmtId="207" fontId="7" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" indent="0"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="7" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="9" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="9" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
+    <x:xf numFmtId="206" fontId="7" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="9" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="9" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
     </x:xf>
     <x:xf numFmtId="203" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" horizontal="left" indent="1"/>
@@ -514,23 +518,23 @@
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" horizontal="center" indent="0"/>
     </x:xf>
-    <x:xf numFmtId="204" fontId="7" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
+    <x:xf numFmtId="207" fontId="7" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" indent="0"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="7" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="9" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="9" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="7" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" horizontal="right" indent="1"/>
+    <x:xf numFmtId="206" fontId="7" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="9" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="9" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="7" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" horizontal="right" indent="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1" horizontal="left" indent="1"/>
@@ -541,20 +545,20 @@
     <x:xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" horizontal="left" indent="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" horizontal="right" indent="1"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="7" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" horizontal="right" indent="1"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" horizontal="right" indent="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" horizontal="right" indent="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" horizontal="right" indent="1"/>
+    <x:xf numFmtId="209" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" horizontal="right" indent="0"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="7" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" horizontal="right" indent="0"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" horizontal="right" indent="0"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="7" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" horizontal="right" indent="0"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" horizontal="right" indent="0"/>
     </x:xf>
     <x:xf numFmtId="203" fontId="7" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1" horizontal="left" indent="1"/>
@@ -565,8 +569,8 @@
     <x:xf numFmtId="200" fontId="7" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1" horizontal="left" indent="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" horizontal="right" indent="1"/>
+    <x:xf numFmtId="209" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" horizontal="right" indent="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" horizontal="left" indent="1"/>
@@ -583,8 +587,8 @@
     <x:xf numFmtId="203" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" horizontal="center" indent="0"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
+    <x:xf numFmtId="208" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" indent="0"/>
@@ -595,14 +599,14 @@
     <x:xf numFmtId="203" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" horizontal="center" indent="0"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="center" indent="1"/>
+    <x:xf numFmtId="208" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" indent="0"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" indent="0"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" horizontal="right" indent="1"/>
+    <x:xf numFmtId="206" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" horizontal="right" indent="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -637,7 +641,7 @@
     <xdr:ext cx="1943100" cy="171858"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="c8ee1591-2c78-4234-bf6f-6135baddbd36"/>
+        <xdr:cNvPr id="1" name="8887580f-7b0f-47b7-b93e-7457b2f70e16"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -675,7 +679,7 @@
     <xdr:ext cx="1943100" cy="171858"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="e01df081-f4b8-4925-affe-ebc20c1374ed"/>
+        <xdr:cNvPr id="1" name="9db8ae8c-daaa-4084-a36d-5fc1af92f140"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -713,7 +717,7 @@
     <xdr:ext cx="1943100" cy="171858"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="bbe9cc96-9a1b-4d8a-821c-e24774918972"/>
+        <xdr:cNvPr id="1" name="545539e7-6733-4b71-8f34-40a7b4497eb7"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -751,7 +755,7 @@
     <xdr:ext cx="1943100" cy="171858"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="a291d147-23eb-4572-9747-8780c272e4a6"/>
+        <xdr:cNvPr id="1" name="8a343158-519e-438a-8d5c-f3c963790dc8"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -1426,7 +1430,7 @@
   <x:headerFooter>
     <x:oddFooter>&amp;L&amp;"UM Sans 2,Regular"&amp;9ULTIMA MILLA S.A. · Uso interno&amp;R&amp;"UM Sans 2,Regular"&amp;9&amp;P / &amp;N</x:oddFooter>
   </x:headerFooter>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra28bef6cb1de41be"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e2fa831a0164b38"/>
 </x:worksheet>
 </file>
 
@@ -2425,7 +2429,7 @@
   <x:headerFooter>
     <x:oddFooter>&amp;L&amp;"UM Sans 2,Regular"&amp;9ULTIMA MILLA S.A. · Uso interno&amp;R&amp;"UM Sans 2,Regular"&amp;9&amp;P / &amp;N</x:oddFooter>
   </x:headerFooter>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc599eb1860ee4425"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a6029e594e346ac"/>
 </x:worksheet>
 </file>
 
@@ -2811,7 +2815,7 @@
   <x:headerFooter>
     <x:oddFooter>&amp;L&amp;"UM Sans 2,Regular"&amp;9ULTIMA MILLA S.A. · Uso interno&amp;R&amp;"UM Sans 2,Regular"&amp;9&amp;P / &amp;N</x:oddFooter>
   </x:headerFooter>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0490fc93e0014d54"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93c65b4c8b9f4a61"/>
 </x:worksheet>
 </file>
 
@@ -3776,6 +3780,6 @@
   <x:headerFooter>
     <x:oddFooter>&amp;L&amp;"UM Sans 2,Regular"&amp;9ULTIMA MILLA S.A. · Uso interno&amp;R&amp;"UM Sans 2,Regular"&amp;9&amp;P / &amp;N</x:oddFooter>
   </x:headerFooter>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re39b6ed7083c4026"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5befd8d4cfcf497d"/>
 </x:worksheet>
 </file>
</xml_diff>